<commit_message>
Scope requested water and sanitation survey to Bo town
</commit_message>
<xml_diff>
--- a/forms/community-water/sl_community_water_service.xlsx
+++ b/forms/community-water/sl_community_water_service.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'survey'!$A$1:$K$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'choices'!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'survey'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'choices'!$A$1:$C$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'settings'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -440,12 +440,13 @@
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +503,11 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>parameters</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>read_only</t>
         </is>
       </c>
     </row>
@@ -525,6 +531,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -546,6 +553,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -560,7 +568,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Sierra Leone community water and sanitation pilot. Explain the purpose and voluntary participation. Do not collect names, phone numbers or personal documents.</t>
+          <t>Bo town water and sanitation pilot. This survey covers Bo town only, not the rest of Bo District. Explain the purpose and voluntary participation. Do not collect names, phone numbers or personal documents.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -571,6 +579,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -600,6 +609,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -629,25 +639,34 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>in_bo_town</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Community water service</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>Is this interview site within Bo town?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Confirm with the respondent or local supervisor. Do not include other towns or villages in Bo District.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>${consent} = 'yes'</t>
@@ -658,90 +677,89 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>select_one interview_unit</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>interview_unit</t>
+          <t>outside_scope</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Reporting unit</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Keep household reports separate from community-representative reports in analysis.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>This site is outside the Bo town survey area. End this interview; do not collect water-service details.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>${consent} = 'yes' and ${in_bo_town} = 'no'</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>visit_date</t>
+          <t>visit</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Visit date</t>
+          <t>Bo town water service</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>${consent} = 'yes' and ${in_bo_town} = 'yes'</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>today()</t>
-        </is>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>select_one district</t>
+          <t>select_one interview_unit</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>interview_unit</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>Reporting unit</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Keep household reports separate from community-representative reports in analysis.</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -753,21 +771,22 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>visit_date</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Town, village or community</t>
+          <t>Visit date</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -777,89 +796,88 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>string-length(.) &lt;= 150</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Use at most 150 characters.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one district</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>site_code</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Water point or community reference</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Use your project reference, for example WASH-0001. Do not use a person’s name.</t>
-        </is>
-      </c>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>regex(., '^[A-Za-z0-9_-]{3,40}$')</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Use 3–40 letters, numbers, underscores or hyphens.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>bo</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>select_one water_source</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>town</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Main drinking-water source</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Bo</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -869,111 +887,126 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>other_source</t>
+          <t>community</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Specify the other source</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>Neighbourhood / section in Bo town</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Use the locally recognized name. Ask the supervisor if uncertain; do not guess a ward number.</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>${water_source} = 'other'</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>string-length(.) &lt;= 150</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Use at most 150 characters.</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>select_one condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>functioning</t>
+          <t>site_code</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Is the main water source functioning today?</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>Water point or site reference</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Use your project reference, for example BO-WASH-0001. Do not use a person’s name.</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>regex(., '^[A-Za-z0-9_-]{3,40}$')</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Use 3–40 letters, numbers, underscores or hyphens.</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one water_source</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>round_trip_minutes</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Reported round-trip time to collect water (minutes)</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Include waiting time. Leave blank if unknown.</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>Main drinking-water source</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 1440</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Enter 0–1,440 minutes.</t>
-        </is>
-      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no_unknown</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>year_round</t>
+          <t>other_source</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Is water reportedly available throughout the year?</t>
+          <t>Specify the other source</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -982,27 +1015,32 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>${water_source} = 'other'</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no_unknown</t>
+          <t>select_one condition</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>safe_storage</t>
+          <t>functioning</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Does the respondent report using a covered water-storage container?</t>
+          <t>Is the main water source functioning today?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1017,35 +1055,45 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>select_one sanitation</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>sanitation</t>
+          <t>round_trip_minutes</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Main sanitation facility used by the community/household interviewed</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>Reported round-trip time to collect water (minutes)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Include waiting time. Leave blank if unknown.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 1440</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Enter 0–1,440 minutes.</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1055,12 +1103,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>handwashing</t>
+          <t>year_round</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Is a handwashing place with water and soap available?</t>
+          <t>Is water reportedly available throughout the year?</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -1075,21 +1123,22 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>select_multiple needs</t>
+          <t>select_one yes_no_unknown</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>priority_needs</t>
+          <t>safe_storage</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Reported priority service needs</t>
+          <t>Does the respondent report using a covered water-storage container?</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1099,34 +1148,27 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>not(selected(., 'none') and count-selected(.) &gt; 1)</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Select None on its own.</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sanitation</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>other_need</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Specify another service need</t>
+          <t>Main sanitation facility used by the community/household interviewed</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1135,38 +1177,31 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>selected(${priority_needs}, 'other')</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>select_one yes_no_unknown</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>location_consent</t>
+          <t>handwashing</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>May the water-point location be recorded?</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Explain that authorized project reviewers can view this location. Refusal does not end the interview.</t>
-        </is>
-      </c>
+          <t>Is a handwashing place with water and soap available?</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1178,158 +1213,270 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>select_multiple needs</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>water_point_location</t>
+          <t>priority_needs</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Optional water-point location</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Record the water point, not a private home. Location accuracy is device-reported.</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>${location_consent} = 'yes'</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Reported priority service needs</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>not(selected(., 'none') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Select None on its own.</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>water_point_photo</t>
+          <t>other_need</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Optional water-point photo</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Obtain permission. Avoid people and personal documents. Leave blank if inappropriate.</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>Specify another service need</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>selected(${priority_needs}, 'other')</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>location_consent</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Observations and limitations</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
+          <t>May the water-point location be recorded?</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Explain that authorized project reviewers can view this location. Refusal does not end the interview.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>string-length(.) &lt;= 1000</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Use at most 1,000 characters.</t>
-        </is>
-      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>interpretation</t>
+          <t>water_point_location</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>This pilot records observations and respondent reports. It does not test water quality or certify safety. Follow your organization’s referral procedure for reported service problems.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>Optional water-point location</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Record the water point, not a private home. Location accuracy is device-reported.</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>${location_consent} = 'yes'</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>water_point_photo</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Optional water-point photo</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Obtain permission. Avoid people and personal documents. Leave blank if inappropriate.</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Observations and limitations</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>string-length(.) &lt;= 1000</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Use at most 1,000 characters.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>This pilot records observations and respondent reports. It does not test water quality or certify safety. Follow your organization’s referral procedure for reported service problems.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K28"/>
+  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1340,7 +1487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1504,736 +1651,481 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>bombali</t>
+          <t>piped</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bombali</t>
+          <t>Piped supply</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>bonthe</t>
+          <t>borehole</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bonthe</t>
+          <t>Borehole / tube well</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>falaba</t>
+          <t>protected_well</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Falaba</t>
+          <t>Protected well</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>kailahun</t>
+          <t>unprotected_well</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Kailahun</t>
+          <t>Unprotected well</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>kambia</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Kambia</t>
+          <t>Spring</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>karene</t>
+          <t>rainwater</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Karene</t>
+          <t>Rainwater</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>kenema</t>
+          <t>surface</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Kenema</t>
+          <t>River, stream, pond or other surface water</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>koinadugu</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Koinadugu</t>
+          <t>Water vendor / tanker</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>kono</t>
+          <t>packaged</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Kono</t>
+          <t>Bottled or sachet water</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>moyamba</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Moyamba</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>port_loko</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Port Loko</t>
+          <t>Functioning</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>pujehun</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pujehun</t>
+          <t>Partly functioning / intermittent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>tonkolili</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Tonkolili</t>
+          <t>Not functioning</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>western_rural</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Western Area Rural</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>western_urban</t>
+          <t>flush</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Western Area Urban</t>
+          <t>Flush or pour-flush toilet</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>piped</t>
+          <t>pit_slab</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Piped supply</t>
+          <t>Pit latrine with slab</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>borehole</t>
+          <t>pit_no_slab</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Borehole / tube well</t>
+          <t>Pit latrine without slab</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>protected_well</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Protected well</t>
+          <t>Shared / communal facility</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>unprotected_well</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Unprotected well</t>
+          <t>No facility</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Spring</t>
+          <t>Other / unknown</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>rainwater</t>
+          <t>repair</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Rainwater</t>
+          <t>Repair the water point</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>surface</t>
+          <t>reliability</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>River, stream, pond or other surface water</t>
+          <t>Improve reliability / seasonal access</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>distance</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Water vendor / tanker</t>
+          <t>Reduce collection distance or waiting time</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>packaged</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Bottled or sachet water</t>
+          <t>Improve storage</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Improve sanitation</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>handwashing</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Functioning</t>
+          <t>Improve handwashing facilities</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Partly functioning / intermittent</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Not functioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>flush</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Flush or pour-flush toilet</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>pit_slab</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Pit latrine with slab</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>pit_no_slab</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Pit latrine without slab</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Shared / communal facility</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>No facility</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Other / unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>repair</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Repair the water point</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>reliability</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Improve reliability / seasonal access</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>distance</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Reduce collection distance or waiting time</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>storage</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Improve storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Improve sanitation</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>handwashing</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Improve handwashing facilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
           <t>None reported</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C52"/>
+  <autoFilter ref="A1:C37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2247,7 +2139,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
@@ -2278,7 +2170,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sierra Leone: Community Water and Sanitation</t>
+          <t>Bo Town: Water and Sanitation</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2288,12 +2180,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026101401</t>
+          <t>2026101402</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>if(${consent} = 'yes', concat(${site_code}, ' - ', ${community}), 'Participation declined')</t>
+          <t>if(${consent} = 'yes', if(${in_bo_town} = 'yes', concat(${site_code}, ' - ', ${community}, ' - Bo'), 'Outside Bo town'), 'Participation declined')</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scope requested water and sanitation survey to Bo town (#116)
</commit_message>
<xml_diff>
--- a/forms/community-water/sl_community_water_service.xlsx
+++ b/forms/community-water/sl_community_water_service.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'survey'!$A$1:$K$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'choices'!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'survey'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'choices'!$A$1:$C$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'settings'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -440,12 +440,13 @@
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +503,11 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>parameters</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>read_only</t>
         </is>
       </c>
     </row>
@@ -525,6 +531,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -546,6 +553,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -560,7 +568,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Sierra Leone community water and sanitation pilot. Explain the purpose and voluntary participation. Do not collect names, phone numbers or personal documents.</t>
+          <t>Bo town water and sanitation pilot. This survey covers Bo town only, not the rest of Bo District. Explain the purpose and voluntary participation. Do not collect names, phone numbers or personal documents.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -571,6 +579,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -600,6 +609,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -629,25 +639,34 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>in_bo_town</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Community water service</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>Is this interview site within Bo town?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Confirm with the respondent or local supervisor. Do not include other towns or villages in Bo District.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>${consent} = 'yes'</t>
@@ -658,90 +677,89 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>select_one interview_unit</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>interview_unit</t>
+          <t>outside_scope</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Reporting unit</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Keep household reports separate from community-representative reports in analysis.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>This site is outside the Bo town survey area. End this interview; do not collect water-service details.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>${consent} = 'yes' and ${in_bo_town} = 'no'</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>visit_date</t>
+          <t>visit</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Visit date</t>
+          <t>Bo town water service</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>${consent} = 'yes' and ${in_bo_town} = 'yes'</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>today()</t>
-        </is>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>select_one district</t>
+          <t>select_one interview_unit</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>interview_unit</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>Reporting unit</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Keep household reports separate from community-representative reports in analysis.</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -753,21 +771,22 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>visit_date</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Town, village or community</t>
+          <t>Visit date</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -777,89 +796,88 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>string-length(.) &lt;= 150</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Use at most 150 characters.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one district</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>site_code</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Water point or community reference</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Use your project reference, for example WASH-0001. Do not use a person’s name.</t>
-        </is>
-      </c>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>regex(., '^[A-Za-z0-9_-]{3,40}$')</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Use 3–40 letters, numbers, underscores or hyphens.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>bo</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>select_one water_source</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>town</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Main drinking-water source</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Bo</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -869,111 +887,126 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>other_source</t>
+          <t>community</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Specify the other source</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>Neighbourhood / section in Bo town</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Use the locally recognized name. Ask the supervisor if uncertain; do not guess a ward number.</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>${water_source} = 'other'</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>string-length(.) &lt;= 150</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Use at most 150 characters.</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>select_one condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>functioning</t>
+          <t>site_code</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Is the main water source functioning today?</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>Water point or site reference</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Use your project reference, for example BO-WASH-0001. Do not use a person’s name.</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>regex(., '^[A-Za-z0-9_-]{3,40}$')</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Use 3–40 letters, numbers, underscores or hyphens.</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one water_source</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>round_trip_minutes</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Reported round-trip time to collect water (minutes)</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Include waiting time. Leave blank if unknown.</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>Main drinking-water source</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 1440</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Enter 0–1,440 minutes.</t>
-        </is>
-      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no_unknown</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>year_round</t>
+          <t>other_source</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Is water reportedly available throughout the year?</t>
+          <t>Specify the other source</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -982,27 +1015,32 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>${water_source} = 'other'</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no_unknown</t>
+          <t>select_one condition</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>safe_storage</t>
+          <t>functioning</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Does the respondent report using a covered water-storage container?</t>
+          <t>Is the main water source functioning today?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1017,35 +1055,45 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>select_one sanitation</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>sanitation</t>
+          <t>round_trip_minutes</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Main sanitation facility used by the community/household interviewed</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>Reported round-trip time to collect water (minutes)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Include waiting time. Leave blank if unknown.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 1440</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Enter 0–1,440 minutes.</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1055,12 +1103,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>handwashing</t>
+          <t>year_round</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Is a handwashing place with water and soap available?</t>
+          <t>Is water reportedly available throughout the year?</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -1075,21 +1123,22 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>select_multiple needs</t>
+          <t>select_one yes_no_unknown</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>priority_needs</t>
+          <t>safe_storage</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Reported priority service needs</t>
+          <t>Does the respondent report using a covered water-storage container?</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1099,34 +1148,27 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>not(selected(., 'none') and count-selected(.) &gt; 1)</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Select None on its own.</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sanitation</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>other_need</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Specify another service need</t>
+          <t>Main sanitation facility used by the community/household interviewed</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1135,38 +1177,31 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>selected(${priority_needs}, 'other')</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>select_one yes_no_unknown</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>location_consent</t>
+          <t>handwashing</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>May the water-point location be recorded?</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Explain that authorized project reviewers can view this location. Refusal does not end the interview.</t>
-        </is>
-      </c>
+          <t>Is a handwashing place with water and soap available?</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1178,158 +1213,270 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>select_multiple needs</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>water_point_location</t>
+          <t>priority_needs</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Optional water-point location</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Record the water point, not a private home. Location accuracy is device-reported.</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>${location_consent} = 'yes'</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Reported priority service needs</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>not(selected(., 'none') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Select None on its own.</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>water_point_photo</t>
+          <t>other_need</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Optional water-point photo</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Obtain permission. Avoid people and personal documents. Leave blank if inappropriate.</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>Specify another service need</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>selected(${priority_needs}, 'other')</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>location_consent</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Observations and limitations</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
+          <t>May the water-point location be recorded?</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Explain that authorized project reviewers can view this location. Refusal does not end the interview.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>string-length(.) &lt;= 1000</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Use at most 1,000 characters.</t>
-        </is>
-      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>interpretation</t>
+          <t>water_point_location</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>This pilot records observations and respondent reports. It does not test water quality or certify safety. Follow your organization’s referral procedure for reported service problems.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>Optional water-point location</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Record the water point, not a private home. Location accuracy is device-reported.</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>${location_consent} = 'yes'</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>water_point_photo</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Optional water-point photo</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Obtain permission. Avoid people and personal documents. Leave blank if inappropriate.</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Observations and limitations</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>string-length(.) &lt;= 1000</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Use at most 1,000 characters.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>This pilot records observations and respondent reports. It does not test water quality or certify safety. Follow your organization’s referral procedure for reported service problems.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K28"/>
+  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1340,7 +1487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1504,736 +1651,481 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>bombali</t>
+          <t>piped</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bombali</t>
+          <t>Piped supply</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>bonthe</t>
+          <t>borehole</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bonthe</t>
+          <t>Borehole / tube well</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>falaba</t>
+          <t>protected_well</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Falaba</t>
+          <t>Protected well</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>kailahun</t>
+          <t>unprotected_well</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Kailahun</t>
+          <t>Unprotected well</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>kambia</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Kambia</t>
+          <t>Spring</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>karene</t>
+          <t>rainwater</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Karene</t>
+          <t>Rainwater</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>kenema</t>
+          <t>surface</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Kenema</t>
+          <t>River, stream, pond or other surface water</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>koinadugu</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Koinadugu</t>
+          <t>Water vendor / tanker</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>kono</t>
+          <t>packaged</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Kono</t>
+          <t>Bottled or sachet water</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>water_source</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>moyamba</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Moyamba</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>port_loko</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Port Loko</t>
+          <t>Functioning</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>pujehun</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pujehun</t>
+          <t>Partly functioning / intermittent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>tonkolili</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Tonkolili</t>
+          <t>Not functioning</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>western_rural</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Western Area Rural</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>western_urban</t>
+          <t>flush</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Western Area Urban</t>
+          <t>Flush or pour-flush toilet</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>piped</t>
+          <t>pit_slab</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Piped supply</t>
+          <t>Pit latrine with slab</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>borehole</t>
+          <t>pit_no_slab</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Borehole / tube well</t>
+          <t>Pit latrine without slab</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>protected_well</t>
+          <t>shared</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Protected well</t>
+          <t>Shared / communal facility</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>unprotected_well</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Unprotected well</t>
+          <t>No facility</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Spring</t>
+          <t>Other / unknown</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>rainwater</t>
+          <t>repair</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Rainwater</t>
+          <t>Repair the water point</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>surface</t>
+          <t>reliability</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>River, stream, pond or other surface water</t>
+          <t>Improve reliability / seasonal access</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>distance</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Water vendor / tanker</t>
+          <t>Reduce collection distance or waiting time</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>packaged</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Bottled or sachet water</t>
+          <t>Improve storage</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>water_source</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>sanitation</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Improve sanitation</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>handwashing</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Functioning</t>
+          <t>Improve handwashing facilities</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Partly functioning / intermittent</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>needs</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Not functioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>flush</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Flush or pour-flush toilet</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>pit_slab</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Pit latrine with slab</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>pit_no_slab</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Pit latrine without slab</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Shared / communal facility</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>No facility</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Other / unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>repair</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Repair the water point</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>reliability</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Improve reliability / seasonal access</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>distance</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Reduce collection distance or waiting time</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>storage</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Improve storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>sanitation</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Improve sanitation</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>handwashing</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Improve handwashing facilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
           <t>None reported</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C52"/>
+  <autoFilter ref="A1:C37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2247,7 +2139,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
@@ -2278,7 +2170,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sierra Leone: Community Water and Sanitation</t>
+          <t>Bo Town: Water and Sanitation</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2288,12 +2180,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026101401</t>
+          <t>2026101402</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>if(${consent} = 'yes', concat(${site_code}, ' - ', ${community}), 'Participation declined')</t>
+          <t>if(${consent} = 'yes', if(${in_bo_town} = 'yes', concat(${site_code}, ' - ', ${community}, ' - Bo'), 'Outside Bo town'), 'Participation declined')</t>
         </is>
       </c>
     </row>

</xml_diff>